<commit_message>
Fix timetable break after 4th period
</commit_message>
<xml_diff>
--- a/school_timetable.xlsx
+++ b/school_timetable.xlsx
@@ -833,11 +833,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>7D COMPUTER</t>
-        </is>
-      </c>
+      <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>9E COMPUTER IX-X</t>
@@ -845,7 +841,11 @@
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr"/>
-      <c r="W2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>7D ISLAMIAT</t>
+        </is>
+      </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
           <t>7B SINDHI</t>
@@ -1010,7 +1010,11 @@
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
       <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>8B GP</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>8A MATHS</t>
@@ -1074,11 +1078,7 @@
       </c>
       <c r="AT3" s="2" t="inlineStr"/>
       <c r="AU3" s="2" t="inlineStr"/>
-      <c r="AV3" s="2" t="inlineStr">
-        <is>
-          <t>8B GAMES</t>
-        </is>
-      </c>
+      <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" s="2" t="inlineStr"/>
       <c r="AX3" s="2" t="inlineStr">
         <is>
@@ -1167,11 +1167,7 @@
           <t>9E COMPUTER IX-X</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>8B S.ST</t>
-        </is>
-      </c>
+      <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr">
@@ -1618,11 +1614,7 @@
           <t>10C CHEMISTRY</t>
         </is>
       </c>
-      <c r="AR7" s="2" t="inlineStr">
-        <is>
-          <t>6B HISTORY</t>
-        </is>
-      </c>
+      <c r="AR7" s="2" t="inlineStr"/>
       <c r="AS7" s="2" t="inlineStr"/>
       <c r="AT7" s="2" t="inlineStr"/>
       <c r="AU7" s="2" t="inlineStr"/>
@@ -1786,12 +1778,12 @@
           <t xml:space="preserve">9F GENERAL SCIENCE </t>
         </is>
       </c>
-      <c r="AR8" s="2" t="inlineStr"/>
-      <c r="AS8" s="2" t="inlineStr">
-        <is>
-          <t>7D SINDHI</t>
-        </is>
-      </c>
+      <c r="AR8" s="2" t="inlineStr">
+        <is>
+          <t>7D S.ST</t>
+        </is>
+      </c>
+      <c r="AS8" s="2" t="inlineStr"/>
       <c r="AT8" s="2" t="inlineStr"/>
       <c r="AU8" s="2" t="inlineStr"/>
       <c r="AV8" s="2" t="inlineStr"/>
@@ -2177,7 +2169,11 @@
           <t>7A GENERAL SCIENCE</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>8B URDU</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
           <t>8C GENERAL SCIENCE</t>
@@ -2215,11 +2211,7 @@
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr">
-        <is>
-          <t>8B S.ST</t>
-        </is>
-      </c>
+      <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="inlineStr">
         <is>
           <t>9E ENGLISH</t>
@@ -3312,11 +3304,7 @@
           <t>9B CHEMISTRY</t>
         </is>
       </c>
-      <c r="AP18" s="2" t="inlineStr">
-        <is>
-          <t>8B MATHS</t>
-        </is>
-      </c>
+      <c r="AP18" s="2" t="inlineStr"/>
       <c r="AQ18" s="2" t="inlineStr"/>
       <c r="AR18" s="2" t="inlineStr">
         <is>
@@ -3326,7 +3314,11 @@
       <c r="AS18" s="2" t="inlineStr"/>
       <c r="AT18" s="2" t="inlineStr"/>
       <c r="AU18" s="2" t="inlineStr"/>
-      <c r="AV18" s="2" t="inlineStr"/>
+      <c r="AV18" s="2" t="inlineStr">
+        <is>
+          <t>8B GAMES</t>
+        </is>
+      </c>
       <c r="AW18" s="2" t="inlineStr">
         <is>
           <t>7B GAMES</t>
@@ -3369,11 +3361,7 @@
           <t>7D GENERAL SCIENCE</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>8B URDU</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr">
@@ -3476,7 +3464,11 @@
           <t>9D CHEMISTRY</t>
         </is>
       </c>
-      <c r="AP19" s="2" t="inlineStr"/>
+      <c r="AP19" s="2" t="inlineStr">
+        <is>
+          <t>8B MATHS</t>
+        </is>
+      </c>
       <c r="AQ19" s="2" t="inlineStr">
         <is>
           <t>10B CHEMISTRY</t>
@@ -3753,11 +3745,7 @@
           <t>9F ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AA21" s="2" t="inlineStr">
-        <is>
-          <t>8B ARABIC</t>
-        </is>
-      </c>
+      <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr">
         <is>
           <t>10D SINDHI-X</t>
@@ -3780,7 +3768,11 @@
         </is>
       </c>
       <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr">
+        <is>
+          <t>8B ISLAMIAT</t>
+        </is>
+      </c>
       <c r="AI21" s="2" t="inlineStr">
         <is>
           <t>10E LIBRARY</t>
@@ -3903,7 +3895,11 @@
           <t>7B COMPUTER</t>
         </is>
       </c>
-      <c r="U22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>8B S.ST</t>
+        </is>
+      </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
           <t>7A ENGLISH</t>
@@ -3944,11 +3940,7 @@
           <t>10F PAKISTAN STUDIES</t>
         </is>
       </c>
-      <c r="AH22" s="2" t="inlineStr">
-        <is>
-          <t>8B ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="AH22" s="2" t="inlineStr"/>
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="inlineStr"/>
       <c r="AK22" s="2" t="inlineStr">
@@ -3986,13 +3978,13 @@
       </c>
       <c r="AT22" s="2" t="inlineStr"/>
       <c r="AU22" s="2" t="inlineStr"/>
-      <c r="AV22" s="2" t="inlineStr">
-        <is>
-          <t>8A GAMES</t>
-        </is>
-      </c>
+      <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" s="2" t="inlineStr"/>
-      <c r="AX22" s="2" t="inlineStr"/>
+      <c r="AX22" s="2" t="inlineStr">
+        <is>
+          <t>8A AI</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr"/>
@@ -4236,7 +4228,11 @@
           <t>9F MATHS</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>6C S.ST</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>7E GENERAL SCIENCE</t>
@@ -4278,7 +4274,11 @@
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>8B COMPUTER</t>
+        </is>
+      </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
           <t>10E ENGLISH</t>
@@ -4297,16 +4297,8 @@
         </is>
       </c>
       <c r="Z25" s="2" t="inlineStr"/>
-      <c r="AA25" s="2" t="inlineStr">
-        <is>
-          <t>6C ISLAMIAT</t>
-        </is>
-      </c>
-      <c r="AB25" s="2" t="inlineStr">
-        <is>
-          <t>8B SINDHI</t>
-        </is>
-      </c>
+      <c r="AA25" s="2" t="inlineStr"/>
+      <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr">
         <is>
           <t>9A MATHS</t>
@@ -4429,7 +4421,11 @@
           <t>6E ENGLISH</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>7D MATHS</t>
+        </is>
+      </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
           <t>6C MATHS</t>
@@ -4443,7 +4439,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>7D COMPUTER</t>
+          <t>8A COMPUTER</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr"/>
@@ -4486,11 +4482,7 @@
           <t>9D MATHS</t>
         </is>
       </c>
-      <c r="AF26" s="2" t="inlineStr">
-        <is>
-          <t>8A GEOGRAPHY</t>
-        </is>
-      </c>
+      <c r="AF26" s="2" t="inlineStr"/>
       <c r="AG26" s="2" t="inlineStr">
         <is>
           <t>8C S.ST</t>
@@ -4609,7 +4601,11 @@
           <t>9F COMPUTER IX-X</t>
         </is>
       </c>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>7D COMPUTER</t>
+        </is>
+      </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
           <t>10F COMPUTER IX-X</t>
@@ -4617,11 +4613,7 @@
       </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="inlineStr"/>
-      <c r="W27" s="2" t="inlineStr">
-        <is>
-          <t>7D ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr">
         <is>
           <t>10A SINDHI-X</t>
@@ -4750,11 +4742,7 @@
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>6A MATHS</t>
-        </is>
-      </c>
+      <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr">
         <is>
           <t>7E URDU</t>
@@ -4800,7 +4788,7 @@
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>8B GP</t>
+          <t>8B SINDHI</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr"/>
@@ -4868,7 +4856,11 @@
       <c r="AU28" s="2" t="inlineStr"/>
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" s="2" t="inlineStr"/>
-      <c r="AX28" s="2" t="inlineStr"/>
+      <c r="AX28" s="2" t="inlineStr">
+        <is>
+          <t>6A AI</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5081,7 +5073,11 @@
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>6E MATHS</t>
+        </is>
+      </c>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr">
         <is>
@@ -5179,11 +5175,7 @@
         </is>
       </c>
       <c r="AR30" s="2" t="inlineStr"/>
-      <c r="AS30" s="2" t="inlineStr">
-        <is>
-          <t>6E SINDHI</t>
-        </is>
-      </c>
+      <c r="AS30" s="2" t="inlineStr"/>
       <c r="AT30" s="2" t="inlineStr"/>
       <c r="AU30" s="2" t="inlineStr"/>
       <c r="AV30" s="2" t="inlineStr">
@@ -5265,11 +5257,7 @@
           <t>7A COMPUTER</t>
         </is>
       </c>
-      <c r="S31" s="2" t="inlineStr">
-        <is>
-          <t>8A COMPUTER</t>
-        </is>
-      </c>
+      <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr">
         <is>
           <t>7C COMPUTER</t>
@@ -5314,7 +5302,11 @@
           <t>10F MATHS</t>
         </is>
       </c>
-      <c r="AF31" s="2" t="inlineStr"/>
+      <c r="AF31" s="2" t="inlineStr">
+        <is>
+          <t>8A GEOGRAPHY</t>
+        </is>
+      </c>
       <c r="AG31" s="2" t="inlineStr"/>
       <c r="AH31" s="2" t="inlineStr">
         <is>
@@ -5417,7 +5409,11 @@
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>7A MATHS</t>
+        </is>
+      </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
           <t>6B MATHS</t>
@@ -5510,25 +5506,21 @@
       </c>
       <c r="AP32" s="2" t="inlineStr"/>
       <c r="AQ32" s="2" t="inlineStr"/>
-      <c r="AR32" s="2" t="inlineStr">
-        <is>
-          <t>7A HISTORY</t>
-        </is>
-      </c>
+      <c r="AR32" s="2" t="inlineStr"/>
       <c r="AS32" s="2" t="inlineStr"/>
       <c r="AT32" s="2" t="inlineStr"/>
       <c r="AU32" s="2" t="inlineStr"/>
-      <c r="AV32" s="2" t="inlineStr"/>
+      <c r="AV32" s="2" t="inlineStr">
+        <is>
+          <t>8A GAMES</t>
+        </is>
+      </c>
       <c r="AW32" s="2" t="inlineStr">
         <is>
           <t>6A GAMES</t>
         </is>
       </c>
-      <c r="AX32" s="2" t="inlineStr">
-        <is>
-          <t>8A AI</t>
-        </is>
-      </c>
+      <c r="AX32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr"/>
@@ -5726,11 +5718,7 @@
           <t xml:space="preserve">9F GENERAL SCIENCE </t>
         </is>
       </c>
-      <c r="AR34" s="2" t="inlineStr">
-        <is>
-          <t>6E S.ST</t>
-        </is>
-      </c>
+      <c r="AR34" s="2" t="inlineStr"/>
       <c r="AS34" s="2" t="inlineStr"/>
       <c r="AT34" s="2" t="inlineStr"/>
       <c r="AU34" s="2" t="inlineStr"/>
@@ -5797,11 +5785,7 @@
           <t>6E ENGLISH</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>7D MATHS</t>
-        </is>
-      </c>
+      <c r="O35" s="2" t="inlineStr"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
           <t>6C MATHS</t>
@@ -5817,12 +5801,12 @@
           <t>8D COMPUTER</t>
         </is>
       </c>
-      <c r="S35" s="2" t="inlineStr"/>
-      <c r="T35" s="2" t="inlineStr">
-        <is>
-          <t>8B COMPUTER</t>
-        </is>
-      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>7D COMPUTER</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr"/>
       <c r="U35" s="2" t="inlineStr">
         <is>
           <t>10E ENGLISH</t>
@@ -5931,11 +5915,7 @@
           <t>10C ENGLISH</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>6D MATHS</t>
-        </is>
-      </c>
+      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>10D PAKISTAN STUDIES</t>
@@ -5977,11 +5957,7 @@
           <t>7B S.ST</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>7D MATHS</t>
-        </is>
-      </c>
+      <c r="O36" s="2" t="inlineStr"/>
       <c r="P36" s="2" t="inlineStr"/>
       <c r="Q36" s="2" t="inlineStr">
         <is>
@@ -6071,11 +6047,19 @@
       <c r="AP36" s="2" t="inlineStr"/>
       <c r="AQ36" s="2" t="inlineStr"/>
       <c r="AR36" s="2" t="inlineStr"/>
-      <c r="AS36" s="2" t="inlineStr"/>
+      <c r="AS36" s="2" t="inlineStr">
+        <is>
+          <t>7D SINDHI</t>
+        </is>
+      </c>
       <c r="AT36" s="2" t="inlineStr"/>
       <c r="AU36" s="2" t="inlineStr"/>
       <c r="AV36" s="2" t="inlineStr"/>
-      <c r="AW36" s="2" t="inlineStr"/>
+      <c r="AW36" s="2" t="inlineStr">
+        <is>
+          <t>6D GAMES</t>
+        </is>
+      </c>
       <c r="AX36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -6259,18 +6243,18 @@
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>6D MATHS</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>6C GENERAL SCIENCE</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>6D URDU</t>
-        </is>
-      </c>
+      <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
@@ -6438,7 +6422,11 @@
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>6D URDU</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>6C ENGLISH</t>
@@ -6461,11 +6449,7 @@
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>6E MATHS</t>
-        </is>
-      </c>
+      <c r="O39" s="2" t="inlineStr"/>
       <c r="P39" s="2" t="inlineStr">
         <is>
           <t>9C MATHS</t>
@@ -6559,15 +6543,15 @@
           <t>7D S.ST</t>
         </is>
       </c>
-      <c r="AS39" s="2" t="inlineStr"/>
+      <c r="AS39" s="2" t="inlineStr">
+        <is>
+          <t>6E SINDHI</t>
+        </is>
+      </c>
       <c r="AT39" s="2" t="inlineStr"/>
       <c r="AU39" s="2" t="inlineStr"/>
       <c r="AV39" s="2" t="inlineStr"/>
-      <c r="AW39" s="2" t="inlineStr">
-        <is>
-          <t>6D GAMES</t>
-        </is>
-      </c>
+      <c r="AW39" s="2" t="inlineStr"/>
       <c r="AX39" s="2" t="inlineStr">
         <is>
           <t>6B AI</t>
@@ -6882,7 +6866,11 @@
           <t>10B CHEMISTRY</t>
         </is>
       </c>
-      <c r="AR41" s="2" t="inlineStr"/>
+      <c r="AR41" s="2" t="inlineStr">
+        <is>
+          <t>6E S.ST</t>
+        </is>
+      </c>
       <c r="AS41" s="2" t="inlineStr">
         <is>
           <t>7E SINDHI</t>
@@ -6895,11 +6883,7 @@
           <t>10F GAMES</t>
         </is>
       </c>
-      <c r="AW41" s="2" t="inlineStr">
-        <is>
-          <t>6E GAMES</t>
-        </is>
-      </c>
+      <c r="AW41" s="2" t="inlineStr"/>
       <c r="AX41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
@@ -6976,11 +6960,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>6C S.ST</t>
-        </is>
-      </c>
+      <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>7E GENERAL SCIENCE</t>
@@ -7023,10 +7003,14 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>7A MATHS</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="inlineStr"/>
+          <t>7D MATHS</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>6C MATHS</t>
+        </is>
+      </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
           <t>9A URDU</t>
@@ -7112,7 +7096,7 @@
       <c r="AQ43" s="2" t="inlineStr"/>
       <c r="AR43" s="2" t="inlineStr">
         <is>
-          <t>7D S.ST</t>
+          <t>7A HISTORY</t>
         </is>
       </c>
       <c r="AS43" s="2" t="inlineStr"/>
@@ -7192,7 +7176,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>6C MATHS</t>
+          <t>6A MATHS</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
@@ -7225,7 +7209,11 @@
       <c r="X44" s="2" t="inlineStr"/>
       <c r="Y44" s="2" t="inlineStr"/>
       <c r="Z44" s="2" t="inlineStr"/>
-      <c r="AA44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>6C ISLAMIAT</t>
+        </is>
+      </c>
       <c r="AB44" s="2" t="inlineStr"/>
       <c r="AC44" s="2" t="inlineStr"/>
       <c r="AD44" s="2" t="inlineStr"/>
@@ -7280,11 +7268,7 @@
       <c r="AU44" s="2" t="inlineStr"/>
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" s="2" t="inlineStr"/>
-      <c r="AX44" s="2" t="inlineStr">
-        <is>
-          <t>6A AI</t>
-        </is>
-      </c>
+      <c r="AX44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed login UI and label visibility
</commit_message>
<xml_diff>
--- a/school_timetable.xlsx
+++ b/school_timetable.xlsx
@@ -498,7 +498,7 @@
     <col width="17" customWidth="1" min="40" max="40"/>
     <col width="17" customWidth="1" min="41" max="41"/>
     <col width="14" customWidth="1" min="42" max="42"/>
-    <col width="23" customWidth="1" min="43" max="43"/>
+    <col width="22" customWidth="1" min="43" max="43"/>
     <col width="19" customWidth="1" min="44" max="44"/>
     <col width="13" customWidth="1" min="45" max="45"/>
     <col width="18" customWidth="1" min="46" max="46"/>
@@ -839,11 +839,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>9C COMPUTER IX-X</t>
-        </is>
-      </c>
+      <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>7C COMPUTER</t>
@@ -882,7 +878,11 @@
           <t>9F ECONOMICS</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>9C ISLAMIAT IX</t>
+        </is>
+      </c>
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
@@ -953,7 +953,11 @@
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>7B ENGLISH</t>
+        </is>
+      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>6B GENERAL SCIENCE</t>
@@ -970,16 +974,8 @@
           <t>8D URDU</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>7B S.ST</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>7D MATHS</t>
-        </is>
-      </c>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="inlineStr"/>
       <c r="Q3" s="3" t="inlineStr"/>
       <c r="R3" s="3" t="inlineStr">
@@ -989,7 +985,7 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>10E COMPUTER IX-X</t>
+          <t>9C COMPUTER IX-X</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
@@ -1027,7 +1023,11 @@
           <t>9A ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr"/>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>7C ISLAMIAT</t>
+        </is>
+      </c>
       <c r="AB3" s="3" t="inlineStr"/>
       <c r="AC3" s="3" t="inlineStr"/>
       <c r="AD3" s="3" t="inlineStr">
@@ -1042,13 +1042,17 @@
         </is>
       </c>
       <c r="AG3" s="3" t="inlineStr"/>
-      <c r="AH3" s="3" t="inlineStr">
-        <is>
-          <t>9C ISLAMIAT IX</t>
-        </is>
-      </c>
-      <c r="AI3" s="3" t="inlineStr"/>
-      <c r="AJ3" s="3" t="inlineStr"/>
+      <c r="AH3" s="3" t="inlineStr"/>
+      <c r="AI3" s="3" t="inlineStr">
+        <is>
+          <t>9B LIBRARY</t>
+        </is>
+      </c>
+      <c r="AJ3" s="3" t="inlineStr">
+        <is>
+          <t>10E PHYSICS</t>
+        </is>
+      </c>
       <c r="AK3" s="3" t="inlineStr">
         <is>
           <t>9D ENGLISH</t>
@@ -1060,11 +1064,7 @@
           <t>10B PHYSICS</t>
         </is>
       </c>
-      <c r="AN3" s="3" t="inlineStr">
-        <is>
-          <t>9B BIOLOGY</t>
-        </is>
-      </c>
+      <c r="AN3" s="3" t="inlineStr"/>
       <c r="AO3" s="3" t="inlineStr">
         <is>
           <t>9E CHEMISTRY</t>
@@ -1072,7 +1072,11 @@
       </c>
       <c r="AP3" s="3" t="inlineStr"/>
       <c r="AQ3" s="3" t="inlineStr"/>
-      <c r="AR3" s="3" t="inlineStr"/>
+      <c r="AR3" s="3" t="inlineStr">
+        <is>
+          <t>7D S.ST</t>
+        </is>
+      </c>
       <c r="AS3" s="3" t="inlineStr"/>
       <c r="AT3" s="3" t="inlineStr"/>
       <c r="AU3" s="3" t="inlineStr"/>
@@ -1081,11 +1085,7 @@
           <t>8A GAMES</t>
         </is>
       </c>
-      <c r="AW3" s="3" t="inlineStr">
-        <is>
-          <t>7C GAMES</t>
-        </is>
-      </c>
+      <c r="AW3" s="3" t="inlineStr"/>
       <c r="AX3" s="3" t="inlineStr">
         <is>
           <t>7A AI</t>
@@ -1137,11 +1137,7 @@
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>9E URDU</t>
-        </is>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr">
@@ -1171,9 +1167,17 @@
           <t>8B ENGLISH</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>7D ISLAMIAT</t>
+        </is>
+      </c>
       <c r="X4" s="2" t="inlineStr"/>
-      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>6E ARABIC</t>
+        </is>
+      </c>
       <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr">
         <is>
@@ -1213,11 +1217,7 @@
       </c>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr"/>
-      <c r="AK4" s="2" t="inlineStr">
-        <is>
-          <t>7C S.ST</t>
-        </is>
-      </c>
+      <c r="AK4" s="2" t="inlineStr"/>
       <c r="AL4" s="2" t="inlineStr">
         <is>
           <t>10B BIOLOGY</t>
@@ -1229,18 +1229,18 @@
           <t>10A CHEMISTRY</t>
         </is>
       </c>
-      <c r="AO4" s="2" t="inlineStr"/>
+      <c r="AO4" s="2" t="inlineStr">
+        <is>
+          <t>9E CHEMISTRY</t>
+        </is>
+      </c>
       <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9F GENERAL SCIENCE </t>
-        </is>
-      </c>
-      <c r="AR4" s="2" t="inlineStr">
-        <is>
-          <t>7D S.ST</t>
-        </is>
-      </c>
+          <t>9F GENERAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="AR4" s="2" t="inlineStr"/>
       <c r="AS4" s="2" t="inlineStr">
         <is>
           <t>6D SINDHI</t>
@@ -1251,7 +1251,7 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" s="2" t="inlineStr">
         <is>
-          <t>6E GAMES</t>
+          <t>7C GAMES</t>
         </is>
       </c>
       <c r="AX4" s="2" t="inlineStr"/>
@@ -1525,7 +1525,11 @@
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>9E URDU</t>
+        </is>
+      </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
           <t>8C ENGLISH</t>
@@ -1548,11 +1552,7 @@
           <t>7D COMPUTER</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>9E COMPUTER IX-X</t>
-        </is>
-      </c>
+      <c r="T7" s="3" t="inlineStr"/>
       <c r="U7" s="3" t="inlineStr">
         <is>
           <t>10B ENGLISH</t>
@@ -1629,14 +1629,14 @@
           <t>6B HISTORY</t>
         </is>
       </c>
-      <c r="AS7" s="3" t="inlineStr"/>
+      <c r="AS7" s="3" t="inlineStr">
+        <is>
+          <t>8D SINDHI</t>
+        </is>
+      </c>
       <c r="AT7" s="3" t="inlineStr"/>
       <c r="AU7" s="3" t="inlineStr"/>
-      <c r="AV7" s="3" t="inlineStr">
-        <is>
-          <t>8D GAMES</t>
-        </is>
-      </c>
+      <c r="AV7" s="3" t="inlineStr"/>
       <c r="AW7" s="3" t="inlineStr"/>
       <c r="AX7" s="3" t="inlineStr"/>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>8A COMPUTER</t>
+          <t>10E COMPUTER IX-X</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
@@ -1916,7 +1916,11 @@
         </is>
       </c>
       <c r="AE9" s="3" t="inlineStr"/>
-      <c r="AF9" s="3" t="inlineStr"/>
+      <c r="AF9" s="3" t="inlineStr">
+        <is>
+          <t>8A GEOGRAPHY</t>
+        </is>
+      </c>
       <c r="AG9" s="3" t="inlineStr">
         <is>
           <t>8D S.ST</t>
@@ -1927,11 +1931,7 @@
           <t>7E PH</t>
         </is>
       </c>
-      <c r="AI9" s="3" t="inlineStr">
-        <is>
-          <t>10E LIBRARY</t>
-        </is>
-      </c>
+      <c r="AI9" s="3" t="inlineStr"/>
       <c r="AJ9" s="3" t="inlineStr">
         <is>
           <t>9E PHYSICS</t>
@@ -1939,11 +1939,7 @@
       </c>
       <c r="AK9" s="3" t="inlineStr"/>
       <c r="AL9" s="3" t="inlineStr"/>
-      <c r="AM9" s="3" t="inlineStr">
-        <is>
-          <t>9A PHYSICS</t>
-        </is>
-      </c>
+      <c r="AM9" s="3" t="inlineStr"/>
       <c r="AN9" s="3" t="inlineStr"/>
       <c r="AO9" s="3" t="inlineStr"/>
       <c r="AP9" s="3" t="inlineStr">
@@ -1962,7 +1958,7 @@
       <c r="AU9" s="3" t="inlineStr"/>
       <c r="AV9" s="3" t="inlineStr">
         <is>
-          <t>9B GAMES</t>
+          <t>9A GAMES</t>
         </is>
       </c>
       <c r="AW9" s="3" t="inlineStr"/>
@@ -2001,11 +1997,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>7B ENGLISH</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2011,11 @@
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>6E TS</t>
+        </is>
+      </c>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
@@ -2029,7 +2025,7 @@
       <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>6E COMPUTER</t>
+          <t>10E COMPUTER IX-X</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
@@ -2053,7 +2049,11 @@
         </is>
       </c>
       <c r="X10" s="2" t="inlineStr"/>
-      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>7B ISLAMIAT</t>
+        </is>
+      </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>6D ISLAMIAT</t>
@@ -2088,11 +2088,7 @@
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr"/>
       <c r="AI10" s="2" t="inlineStr"/>
-      <c r="AJ10" s="2" t="inlineStr">
-        <is>
-          <t>10E PHYSICS</t>
-        </is>
-      </c>
+      <c r="AJ10" s="2" t="inlineStr"/>
       <c r="AK10" s="2" t="inlineStr">
         <is>
           <t>10D ENGLISH</t>
@@ -2397,7 +2393,7 @@
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>7C ISLAMIAT</t>
+          <t>7C ARABIC</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
@@ -2507,11 +2503,7 @@
       </c>
       <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="3" t="inlineStr"/>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>6E TS</t>
-        </is>
-      </c>
+      <c r="O13" s="3" t="inlineStr"/>
       <c r="P13" s="3" t="inlineStr"/>
       <c r="Q13" s="3" t="inlineStr"/>
       <c r="R13" s="3" t="inlineStr">
@@ -2540,17 +2532,9 @@
           <t>8A ISLAMIAT</t>
         </is>
       </c>
-      <c r="X13" s="3" t="inlineStr">
-        <is>
-          <t>10C SINDHI-X</t>
-        </is>
-      </c>
+      <c r="X13" s="3" t="inlineStr"/>
       <c r="Y13" s="3" t="inlineStr"/>
-      <c r="Z13" s="3" t="inlineStr">
-        <is>
-          <t>9A ISLAMIAT IX</t>
-        </is>
-      </c>
+      <c r="Z13" s="3" t="inlineStr"/>
       <c r="AA13" s="3" t="inlineStr">
         <is>
           <t>6C ISLAMIAT</t>
@@ -2606,8 +2590,16 @@
           <t>9B CHEMISTRY</t>
         </is>
       </c>
-      <c r="AP13" s="3" t="inlineStr"/>
-      <c r="AQ13" s="3" t="inlineStr"/>
+      <c r="AP13" s="3" t="inlineStr">
+        <is>
+          <t>10C MATHS</t>
+        </is>
+      </c>
+      <c r="AQ13" s="3" t="inlineStr">
+        <is>
+          <t>9A CHEMISTRY</t>
+        </is>
+      </c>
       <c r="AR13" s="3" t="inlineStr">
         <is>
           <t>6B HISTORY</t>
@@ -2625,7 +2617,11 @@
           <t>10B GAMES</t>
         </is>
       </c>
-      <c r="AW13" s="3" t="inlineStr"/>
+      <c r="AW13" s="3" t="inlineStr">
+        <is>
+          <t>6E GAMES</t>
+        </is>
+      </c>
       <c r="AX13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
@@ -2907,11 +2903,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>8A COMPUTER</t>
-        </is>
-      </c>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr">
         <is>
@@ -2934,7 +2926,11 @@
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>9A ISLAMIAT IX</t>
+        </is>
+      </c>
       <c r="AA16" s="2" t="inlineStr">
         <is>
           <t>6B ISLAMIAT</t>
@@ -2962,15 +2958,19 @@
         </is>
       </c>
       <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AH16" s="2" t="inlineStr">
+        <is>
+          <t>7D PH</t>
+        </is>
+      </c>
       <c r="AI16" s="2" t="inlineStr"/>
-      <c r="AJ16" s="2" t="inlineStr"/>
+      <c r="AJ16" s="2" t="inlineStr">
+        <is>
+          <t>10E PHYSICS</t>
+        </is>
+      </c>
       <c r="AK16" s="2" t="inlineStr"/>
-      <c r="AL16" s="2" t="inlineStr">
-        <is>
-          <t>9A BIOLOGY</t>
-        </is>
-      </c>
+      <c r="AL16" s="2" t="inlineStr"/>
       <c r="AM16" s="2" t="inlineStr">
         <is>
           <t>10C PHYSICS</t>
@@ -2989,14 +2989,10 @@
       </c>
       <c r="AQ16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9F GENERAL SCIENCE </t>
-        </is>
-      </c>
-      <c r="AR16" s="2" t="inlineStr">
-        <is>
-          <t>7D S.ST</t>
-        </is>
-      </c>
+          <t>9F GENERAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="AR16" s="2" t="inlineStr"/>
       <c r="AS16" s="2" t="inlineStr">
         <is>
           <t>7E SINDHI</t>
@@ -3004,13 +3000,13 @@
       </c>
       <c r="AT16" s="2" t="inlineStr"/>
       <c r="AU16" s="2" t="inlineStr"/>
-      <c r="AV16" s="2" t="inlineStr">
-        <is>
-          <t>10E GAMES</t>
-        </is>
-      </c>
+      <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" s="2" t="inlineStr"/>
-      <c r="AX16" s="2" t="inlineStr"/>
+      <c r="AX16" s="2" t="inlineStr">
+        <is>
+          <t>8A AI</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr"/>
@@ -3123,25 +3119,25 @@
         </is>
       </c>
       <c r="AH17" s="3" t="inlineStr"/>
-      <c r="AI17" s="3" t="inlineStr">
-        <is>
-          <t>9B LIBRARY</t>
-        </is>
-      </c>
+      <c r="AI17" s="3" t="inlineStr"/>
       <c r="AJ17" s="3" t="inlineStr"/>
-      <c r="AK17" s="3" t="inlineStr"/>
+      <c r="AK17" s="3" t="inlineStr">
+        <is>
+          <t>7C S.ST</t>
+        </is>
+      </c>
       <c r="AL17" s="3" t="inlineStr"/>
       <c r="AM17" s="3" t="inlineStr">
         <is>
           <t>10A PHYSICS</t>
         </is>
       </c>
-      <c r="AN17" s="3" t="inlineStr"/>
-      <c r="AO17" s="3" t="inlineStr">
-        <is>
-          <t>9E CHEMISTRY</t>
-        </is>
-      </c>
+      <c r="AN17" s="3" t="inlineStr">
+        <is>
+          <t>9B BIOLOGY</t>
+        </is>
+      </c>
+      <c r="AO17" s="3" t="inlineStr"/>
       <c r="AP17" s="3" t="inlineStr">
         <is>
           <t>10C MATHS</t>
@@ -3157,14 +3153,14 @@
           <t>8A HISTORY</t>
         </is>
       </c>
-      <c r="AS17" s="3" t="inlineStr">
-        <is>
-          <t>7C SINDHI</t>
-        </is>
-      </c>
+      <c r="AS17" s="3" t="inlineStr"/>
       <c r="AT17" s="3" t="inlineStr"/>
       <c r="AU17" s="3" t="inlineStr"/>
-      <c r="AV17" s="3" t="inlineStr"/>
+      <c r="AV17" s="3" t="inlineStr">
+        <is>
+          <t>9E GAMES</t>
+        </is>
+      </c>
       <c r="AW17" s="3" t="inlineStr">
         <is>
           <t>6B GAMES</t>
@@ -3694,11 +3690,7 @@
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>6B GENERAL SCIENCE</t>
-        </is>
-      </c>
+      <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="3" t="inlineStr"/>
       <c r="L21" s="3" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr">
@@ -3738,7 +3730,11 @@
           <t>10F ENGLISH</t>
         </is>
       </c>
-      <c r="V21" s="3" t="inlineStr"/>
+      <c r="V21" s="3" t="inlineStr">
+        <is>
+          <t>9F ENGLISH</t>
+        </is>
+      </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
           <t>8D ARABIC</t>
@@ -3780,11 +3776,7 @@
           <t>10B LIBRARY</t>
         </is>
       </c>
-      <c r="AJ21" s="3" t="inlineStr">
-        <is>
-          <t>10E PHYSICS</t>
-        </is>
-      </c>
+      <c r="AJ21" s="3" t="inlineStr"/>
       <c r="AK21" s="3" t="inlineStr">
         <is>
           <t>7C S.ST</t>
@@ -3795,11 +3787,7 @@
           <t>10A BIOLOGY</t>
         </is>
       </c>
-      <c r="AM21" s="3" t="inlineStr">
-        <is>
-          <t>10C PHYSICS</t>
-        </is>
-      </c>
+      <c r="AM21" s="3" t="inlineStr"/>
       <c r="AN21" s="3" t="inlineStr">
         <is>
           <t>9B BIOLOGY</t>
@@ -3817,10 +3805,14 @@
       </c>
       <c r="AQ21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9F GENERAL SCIENCE </t>
-        </is>
-      </c>
-      <c r="AR21" s="3" t="inlineStr"/>
+          <t>10E CHEMISTRY</t>
+        </is>
+      </c>
+      <c r="AR21" s="3" t="inlineStr">
+        <is>
+          <t>6B GEOGRAPHY</t>
+        </is>
+      </c>
       <c r="AS21" s="3" t="inlineStr"/>
       <c r="AT21" s="3" t="inlineStr"/>
       <c r="AU21" s="3" t="inlineStr"/>
@@ -3855,7 +3847,11 @@
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>8D GENERAL SCIENCE</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>7A URDU</t>
@@ -3877,11 +3873,7 @@
           <t>6E GENERAL SCIENCE</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>8D URDU</t>
-        </is>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
           <t>6B ENGLISH</t>
@@ -3903,11 +3895,7 @@
           <t>9F COMPUTER IX-X</t>
         </is>
       </c>
-      <c r="S22" s="2" t="inlineStr">
-        <is>
-          <t>10E COMPUTER IX-X</t>
-        </is>
-      </c>
+      <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr">
         <is>
           <t>9E COMPUTER IX-X</t>
@@ -3963,7 +3951,11 @@
         </is>
       </c>
       <c r="AH22" s="2" t="inlineStr"/>
-      <c r="AI22" s="2" t="inlineStr"/>
+      <c r="AI22" s="2" t="inlineStr">
+        <is>
+          <t>10E LIBRARY</t>
+        </is>
+      </c>
       <c r="AJ22" s="2" t="inlineStr"/>
       <c r="AK22" s="2" t="inlineStr"/>
       <c r="AL22" s="2" t="inlineStr"/>
@@ -4074,7 +4066,7 @@
       <c r="S23" s="3" t="inlineStr"/>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>6B COMPUTER</t>
+          <t>9E COMPUTER IX-X</t>
         </is>
       </c>
       <c r="U23" s="3" t="inlineStr"/>
@@ -4095,11 +4087,7 @@
           <t>9A ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AA23" s="3" t="inlineStr">
-        <is>
-          <t>7C ARABIC</t>
-        </is>
-      </c>
+      <c r="AA23" s="3" t="inlineStr"/>
       <c r="AB23" s="3" t="inlineStr">
         <is>
           <t>10D SINDHI-X</t>
@@ -4153,16 +4141,20 @@
       </c>
       <c r="AQ23" s="3" t="inlineStr"/>
       <c r="AR23" s="3" t="inlineStr"/>
-      <c r="AS23" s="3" t="inlineStr"/>
+      <c r="AS23" s="3" t="inlineStr">
+        <is>
+          <t>7C SINDHI</t>
+        </is>
+      </c>
       <c r="AT23" s="3" t="inlineStr"/>
       <c r="AU23" s="3" t="inlineStr"/>
-      <c r="AV23" s="3" t="inlineStr">
-        <is>
-          <t>9E GAMES</t>
-        </is>
-      </c>
+      <c r="AV23" s="3" t="inlineStr"/>
       <c r="AW23" s="3" t="inlineStr"/>
-      <c r="AX23" s="3" t="inlineStr"/>
+      <c r="AX23" s="3" t="inlineStr">
+        <is>
+          <t>6B AI</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr"/>
@@ -4232,25 +4224,29 @@
           <t>11:20-12:00</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>10C ENGLISH</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
           <t>9B MATHS</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>8D GENERAL SCIENCE</t>
-        </is>
-      </c>
+      <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr">
         <is>
           <t>6D URDU</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>6B GENERAL SCIENCE</t>
+        </is>
+      </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>9C URDU</t>
@@ -4286,11 +4282,7 @@
         </is>
       </c>
       <c r="U25" s="3" t="inlineStr"/>
-      <c r="V25" s="3" t="inlineStr">
-        <is>
-          <t>9F ENGLISH</t>
-        </is>
-      </c>
+      <c r="V25" s="3" t="inlineStr"/>
       <c r="W25" s="3" t="inlineStr">
         <is>
           <t>7D ARABIC</t>
@@ -4336,7 +4328,11 @@
           <t>9A LIBRARY</t>
         </is>
       </c>
-      <c r="AJ25" s="3" t="inlineStr"/>
+      <c r="AJ25" s="3" t="inlineStr">
+        <is>
+          <t>10E PHYSICS</t>
+        </is>
+      </c>
       <c r="AK25" s="3" t="inlineStr"/>
       <c r="AL25" s="3" t="inlineStr">
         <is>
@@ -4357,7 +4353,7 @@
       </c>
       <c r="AQ25" s="3" t="inlineStr">
         <is>
-          <t>10E CHEMISTRY</t>
+          <t>9F GENERAL SCIENCE</t>
         </is>
       </c>
       <c r="AR25" s="3" t="inlineStr">
@@ -4374,15 +4370,11 @@
       <c r="AU25" s="3" t="inlineStr"/>
       <c r="AV25" s="3" t="inlineStr">
         <is>
-          <t>10C GAMES</t>
+          <t>8D GAMES</t>
         </is>
       </c>
       <c r="AW25" s="3" t="inlineStr"/>
-      <c r="AX25" s="3" t="inlineStr">
-        <is>
-          <t>6B AI</t>
-        </is>
-      </c>
+      <c r="AX25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr"/>
@@ -4464,7 +4456,11 @@
           <t>8D ISLAMIAT</t>
         </is>
       </c>
-      <c r="X26" s="2" t="inlineStr"/>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>10C SINDHI-X</t>
+        </is>
+      </c>
       <c r="Y26" s="2" t="inlineStr">
         <is>
           <t>6E ARABIC</t>
@@ -4526,11 +4522,7 @@
           <t>9E CHEMISTRY</t>
         </is>
       </c>
-      <c r="AP26" s="2" t="inlineStr">
-        <is>
-          <t>10C MATHS</t>
-        </is>
-      </c>
+      <c r="AP26" s="2" t="inlineStr"/>
       <c r="AQ26" s="2" t="inlineStr"/>
       <c r="AR26" s="2" t="inlineStr">
         <is>
@@ -4724,11 +4716,7 @@
           <t>1:20-2:00</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>10C ENGLISH</t>
-        </is>
-      </c>
+      <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>7B MATHS</t>
@@ -4761,7 +4749,11 @@
           <t xml:space="preserve">10F GENERAL SCIENCE </t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>8D URDU</t>
+        </is>
+      </c>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -4817,17 +4809,17 @@
           <t>8A GEOGRAPHY</t>
         </is>
       </c>
-      <c r="AG28" s="2" t="inlineStr">
-        <is>
-          <t>8D S.ST</t>
-        </is>
-      </c>
+      <c r="AG28" s="2" t="inlineStr"/>
       <c r="AH28" s="2" t="inlineStr">
         <is>
           <t>9E ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AI28" s="2" t="inlineStr"/>
+      <c r="AI28" s="2" t="inlineStr">
+        <is>
+          <t>10C LIBRARY</t>
+        </is>
+      </c>
       <c r="AJ28" s="2" t="inlineStr"/>
       <c r="AK28" s="2" t="inlineStr"/>
       <c r="AL28" s="2" t="inlineStr">
@@ -4939,7 +4931,11 @@
           <t>7E ENGLISH</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>7D MATHS</t>
+        </is>
+      </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
           <t>6B MATHS</t>
@@ -4998,11 +4994,7 @@
           <t>9F ECONOMICS</t>
         </is>
       </c>
-      <c r="AH29" s="3" t="inlineStr">
-        <is>
-          <t>7D PH</t>
-        </is>
-      </c>
+      <c r="AH29" s="3" t="inlineStr"/>
       <c r="AI29" s="3" t="inlineStr"/>
       <c r="AJ29" s="3" t="inlineStr">
         <is>
@@ -5106,11 +5098,7 @@
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>8D COMPUTER</t>
-        </is>
-      </c>
+      <c r="R30" s="2" t="inlineStr"/>
       <c r="S30" s="2" t="inlineStr">
         <is>
           <t>10E COMPUTER IX-X</t>
@@ -5145,18 +5133,18 @@
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>10A MATHS</t>
+        </is>
+      </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
           <t>7C MATHS</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr"/>
-      <c r="AF30" s="2" t="inlineStr">
-        <is>
-          <t>10A PAKISTAN STUDIES</t>
-        </is>
-      </c>
+      <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr">
         <is>
           <t>8C S.ST</t>
@@ -5174,7 +5162,11 @@
         </is>
       </c>
       <c r="AK30" s="2" t="inlineStr"/>
-      <c r="AL30" s="2" t="inlineStr"/>
+      <c r="AL30" s="2" t="inlineStr">
+        <is>
+          <t>9A BIOLOGY</t>
+        </is>
+      </c>
       <c r="AM30" s="2" t="inlineStr">
         <is>
           <t>10C PHYSICS</t>
@@ -5197,14 +5189,14 @@
           <t>8A HISTORY</t>
         </is>
       </c>
-      <c r="AS30" s="2" t="inlineStr"/>
+      <c r="AS30" s="2" t="inlineStr">
+        <is>
+          <t>8D SINDHI</t>
+        </is>
+      </c>
       <c r="AT30" s="2" t="inlineStr"/>
       <c r="AU30" s="2" t="inlineStr"/>
-      <c r="AV30" s="2" t="inlineStr">
-        <is>
-          <t>9A GAMES</t>
-        </is>
-      </c>
+      <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" s="2" t="inlineStr"/>
       <c r="AX30" s="2" t="inlineStr"/>
     </row>
@@ -5308,18 +5300,18 @@
           <t>10F MATHS</t>
         </is>
       </c>
-      <c r="AF31" s="3" t="inlineStr"/>
+      <c r="AF31" s="3" t="inlineStr">
+        <is>
+          <t>10A PAKISTAN STUDIES</t>
+        </is>
+      </c>
       <c r="AG31" s="3" t="inlineStr"/>
       <c r="AH31" s="3" t="inlineStr">
         <is>
           <t>9E ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AI31" s="3" t="inlineStr">
-        <is>
-          <t>10C LIBRARY</t>
-        </is>
-      </c>
+      <c r="AI31" s="3" t="inlineStr"/>
       <c r="AJ31" s="3" t="inlineStr">
         <is>
           <t>10E PHYSICS</t>
@@ -5333,7 +5325,7 @@
       <c r="AL31" s="3" t="inlineStr"/>
       <c r="AM31" s="3" t="inlineStr">
         <is>
-          <t>10A PHYSICS</t>
+          <t>10C PHYSICS</t>
         </is>
       </c>
       <c r="AN31" s="3" t="inlineStr">
@@ -5352,11 +5344,7 @@
           <t>9A CHEMISTRY</t>
         </is>
       </c>
-      <c r="AR31" s="3" t="inlineStr">
-        <is>
-          <t>6A HISTORY</t>
-        </is>
-      </c>
+      <c r="AR31" s="3" t="inlineStr"/>
       <c r="AS31" s="3" t="inlineStr">
         <is>
           <t>6E SINDHI</t>
@@ -5370,7 +5358,11 @@
         </is>
       </c>
       <c r="AW31" s="3" t="inlineStr"/>
-      <c r="AX31" s="3" t="inlineStr"/>
+      <c r="AX31" s="3" t="inlineStr">
+        <is>
+          <t>6A AI</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr"/>
@@ -5412,7 +5404,11 @@
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>6E GENERAL SCIENCE</t>
+        </is>
+      </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
           <t>9F URDU</t>
@@ -5457,11 +5453,7 @@
           <t>10A SINDHI-X</t>
         </is>
       </c>
-      <c r="Y32" s="2" t="inlineStr">
-        <is>
-          <t>6E ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="Y32" s="2" t="inlineStr"/>
       <c r="Z32" s="2" t="inlineStr">
         <is>
           <t>6D ARABIC</t>
@@ -5626,24 +5618,24 @@
           <t>6C ENGLISH</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>6B GENERAL SCIENCE</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>9B URDU</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>6E GENERAL SCIENCE</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>7D MATHS</t>
-        </is>
-      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>7B S.ST</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
           <t>9C MATHS</t>
@@ -5655,7 +5647,11 @@
           <t>8C COMPUTER</t>
         </is>
       </c>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>6E COMPUTER</t>
+        </is>
+      </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
           <t>10F COMPUTER IX-X</t>
@@ -5681,11 +5677,7 @@
           <t>10E SINDHI-X</t>
         </is>
       </c>
-      <c r="Y34" s="2" t="inlineStr">
-        <is>
-          <t>7B ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="Y34" s="2" t="inlineStr"/>
       <c r="Z34" s="2" t="inlineStr">
         <is>
           <t>9F ISLAMIAT IX</t>
@@ -5705,7 +5697,11 @@
       </c>
       <c r="AE34" s="2" t="inlineStr"/>
       <c r="AF34" s="2" t="inlineStr"/>
-      <c r="AG34" s="2" t="inlineStr"/>
+      <c r="AG34" s="2" t="inlineStr">
+        <is>
+          <t>8D S.ST</t>
+        </is>
+      </c>
       <c r="AH34" s="2" t="inlineStr">
         <is>
           <t>8B ISLAMIAT</t>
@@ -5734,14 +5730,10 @@
       <c r="AQ34" s="2" t="inlineStr"/>
       <c r="AR34" s="2" t="inlineStr">
         <is>
-          <t>6B GEOGRAPHY</t>
-        </is>
-      </c>
-      <c r="AS34" s="2" t="inlineStr">
-        <is>
-          <t>8D SINDHI</t>
-        </is>
-      </c>
+          <t>7D S.ST</t>
+        </is>
+      </c>
+      <c r="AS34" s="2" t="inlineStr"/>
       <c r="AT34" s="2" t="inlineStr"/>
       <c r="AU34" s="2" t="inlineStr"/>
       <c r="AV34" s="2" t="inlineStr">
@@ -5768,7 +5760,11 @@
           <t>12:10-12:45</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>7D ENGLISH</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
           <t>7B MATHS</t>
@@ -5782,11 +5778,7 @@
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>6B GENERAL SCIENCE</t>
-        </is>
-      </c>
+      <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -5819,8 +5811,16 @@
           <t>6A COMPUTER</t>
         </is>
       </c>
-      <c r="S35" s="3" t="inlineStr"/>
-      <c r="T35" s="3" t="inlineStr"/>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>8A COMPUTER</t>
+        </is>
+      </c>
+      <c r="T35" s="3" t="inlineStr">
+        <is>
+          <t>6B COMPUTER</t>
+        </is>
+      </c>
       <c r="U35" s="3" t="inlineStr"/>
       <c r="V35" s="3" t="inlineStr"/>
       <c r="W35" s="3" t="inlineStr">
@@ -5863,11 +5863,7 @@
           <t>9B ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AI35" s="3" t="inlineStr">
-        <is>
-          <t>10A LIBRARY</t>
-        </is>
-      </c>
+      <c r="AI35" s="3" t="inlineStr"/>
       <c r="AJ35" s="3" t="inlineStr">
         <is>
           <t>9E PHYSICS</t>
@@ -5884,7 +5880,11 @@
           <t>9C PHYSICS</t>
         </is>
       </c>
-      <c r="AN35" s="3" t="inlineStr"/>
+      <c r="AN35" s="3" t="inlineStr">
+        <is>
+          <t>10A CHEMISTRY</t>
+        </is>
+      </c>
       <c r="AO35" s="3" t="inlineStr">
         <is>
           <t>9D CHEMISTRY</t>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="AQ35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9F GENERAL SCIENCE </t>
+          <t>9F GENERAL SCIENCE</t>
         </is>
       </c>
       <c r="AR35" s="3" t="inlineStr"/>
@@ -5909,16 +5909,8 @@
       <c r="AT35" s="3" t="inlineStr"/>
       <c r="AU35" s="3" t="inlineStr"/>
       <c r="AV35" s="3" t="inlineStr"/>
-      <c r="AW35" s="3" t="inlineStr">
-        <is>
-          <t>7D GAMES</t>
-        </is>
-      </c>
-      <c r="AX35" s="3" t="inlineStr">
-        <is>
-          <t>8A AI</t>
-        </is>
-      </c>
+      <c r="AW35" s="3" t="inlineStr"/>
+      <c r="AX35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr"/>
@@ -6096,11 +6088,7 @@
           <t>1:15-2:00</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>7D ENGLISH</t>
-        </is>
-      </c>
+      <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
@@ -6151,11 +6139,7 @@
         </is>
       </c>
       <c r="R37" s="3" t="inlineStr"/>
-      <c r="S37" s="3" t="inlineStr">
-        <is>
-          <t>8A COMPUTER</t>
-        </is>
-      </c>
+      <c r="S37" s="3" t="inlineStr"/>
       <c r="T37" s="3" t="inlineStr"/>
       <c r="U37" s="3" t="inlineStr">
         <is>
@@ -6167,11 +6151,15 @@
           <t>9F ENGLISH</t>
         </is>
       </c>
-      <c r="W37" s="3" t="inlineStr"/>
+      <c r="W37" s="3" t="inlineStr">
+        <is>
+          <t>8A ARABIC</t>
+        </is>
+      </c>
       <c r="X37" s="3" t="inlineStr"/>
       <c r="Y37" s="3" t="inlineStr">
         <is>
-          <t>6E ARABIC</t>
+          <t>6E ISLAMIAT</t>
         </is>
       </c>
       <c r="Z37" s="3" t="inlineStr"/>
@@ -6211,12 +6199,12 @@
         </is>
       </c>
       <c r="AL37" s="3" t="inlineStr"/>
-      <c r="AM37" s="3" t="inlineStr"/>
-      <c r="AN37" s="3" t="inlineStr">
-        <is>
-          <t>10A CHEMISTRY</t>
-        </is>
-      </c>
+      <c r="AM37" s="3" t="inlineStr">
+        <is>
+          <t>10A PHYSICS</t>
+        </is>
+      </c>
+      <c r="AN37" s="3" t="inlineStr"/>
       <c r="AO37" s="3" t="inlineStr">
         <is>
           <t>9B PHYSICS</t>
@@ -6245,7 +6233,11 @@
       <c r="AT37" s="3" t="inlineStr"/>
       <c r="AU37" s="3" t="inlineStr"/>
       <c r="AV37" s="3" t="inlineStr"/>
-      <c r="AW37" s="3" t="inlineStr"/>
+      <c r="AW37" s="3" t="inlineStr">
+        <is>
+          <t>7D GAMES</t>
+        </is>
+      </c>
       <c r="AX37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -6286,7 +6278,11 @@
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>7D GENERAL SCIENCE</t>
+        </is>
+      </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
           <t>9C URDU</t>
@@ -6321,7 +6317,7 @@
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>6E COMPUTER</t>
+          <t>8A COMPUTER</t>
         </is>
       </c>
       <c r="T38" s="2" t="inlineStr"/>
@@ -6331,11 +6327,7 @@
           <t>9E ENGLISH</t>
         </is>
       </c>
-      <c r="W38" s="2" t="inlineStr">
-        <is>
-          <t>7D ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="W38" s="2" t="inlineStr"/>
       <c r="X38" s="2" t="inlineStr">
         <is>
           <t>10E SINDHI-X</t>
@@ -6372,11 +6364,7 @@
           <t>10F MATHS</t>
         </is>
       </c>
-      <c r="AF38" s="2" t="inlineStr">
-        <is>
-          <t>8A GEOGRAPHY</t>
-        </is>
-      </c>
+      <c r="AF38" s="2" t="inlineStr"/>
       <c r="AG38" s="2" t="inlineStr">
         <is>
           <t>9F ECONOMICS</t>
@@ -6409,7 +6397,11 @@
           <t>6B GEOGRAPHY</t>
         </is>
       </c>
-      <c r="AS38" s="2" t="inlineStr"/>
+      <c r="AS38" s="2" t="inlineStr">
+        <is>
+          <t>6E SINDHI</t>
+        </is>
+      </c>
       <c r="AT38" s="2" t="inlineStr"/>
       <c r="AU38" s="2" t="inlineStr"/>
       <c r="AV38" s="2" t="inlineStr"/>
@@ -6483,7 +6475,11 @@
         </is>
       </c>
       <c r="R39" s="3" t="inlineStr"/>
-      <c r="S39" s="3" t="inlineStr"/>
+      <c r="S39" s="3" t="inlineStr">
+        <is>
+          <t>6E COMPUTER</t>
+        </is>
+      </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
           <t>6B COMPUTER</t>
@@ -6517,11 +6513,7 @@
           <t>10F SINDHI-X</t>
         </is>
       </c>
-      <c r="AC39" s="3" t="inlineStr">
-        <is>
-          <t>10A MATHS</t>
-        </is>
-      </c>
+      <c r="AC39" s="3" t="inlineStr"/>
       <c r="AD39" s="3" t="inlineStr">
         <is>
           <t>9D PHYSICS</t>
@@ -6543,7 +6535,11 @@
           <t>9C ISLAMIAT IX</t>
         </is>
       </c>
-      <c r="AI39" s="3" t="inlineStr"/>
+      <c r="AI39" s="3" t="inlineStr">
+        <is>
+          <t>10A LIBRARY</t>
+        </is>
+      </c>
       <c r="AJ39" s="3" t="inlineStr"/>
       <c r="AK39" s="3" t="inlineStr"/>
       <c r="AL39" s="3" t="inlineStr"/>
@@ -6569,11 +6565,7 @@
           <t>8A HISTORY</t>
         </is>
       </c>
-      <c r="AS39" s="3" t="inlineStr">
-        <is>
-          <t>6E SINDHI</t>
-        </is>
-      </c>
+      <c r="AS39" s="3" t="inlineStr"/>
       <c r="AT39" s="3" t="inlineStr"/>
       <c r="AU39" s="3" t="inlineStr"/>
       <c r="AV39" s="3" t="inlineStr"/>
@@ -6646,7 +6638,11 @@
           <t>9D URDU</t>
         </is>
       </c>
-      <c r="R40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>8D COMPUTER</t>
+        </is>
+      </c>
       <c r="S40" s="2" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
@@ -6700,11 +6696,7 @@
       </c>
       <c r="AH40" s="2" t="inlineStr"/>
       <c r="AI40" s="2" t="inlineStr"/>
-      <c r="AJ40" s="2" t="inlineStr">
-        <is>
-          <t>10E PHYSICS</t>
-        </is>
-      </c>
+      <c r="AJ40" s="2" t="inlineStr"/>
       <c r="AK40" s="2" t="inlineStr">
         <is>
           <t>10A ENGLISH</t>
@@ -6733,14 +6725,14 @@
         </is>
       </c>
       <c r="AR40" s="2" t="inlineStr"/>
-      <c r="AS40" s="2" t="inlineStr">
-        <is>
-          <t>8D SINDHI</t>
-        </is>
-      </c>
+      <c r="AS40" s="2" t="inlineStr"/>
       <c r="AT40" s="2" t="inlineStr"/>
       <c r="AU40" s="2" t="inlineStr"/>
-      <c r="AV40" s="2" t="inlineStr"/>
+      <c r="AV40" s="2" t="inlineStr">
+        <is>
+          <t>10E GAMES</t>
+        </is>
+      </c>
       <c r="AW40" s="2" t="inlineStr"/>
       <c r="AX40" s="2" t="inlineStr"/>
     </row>
@@ -6778,11 +6770,7 @@
           <t>6D ENGLISH</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>7D GENERAL SCIENCE</t>
-        </is>
-      </c>
+      <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
           <t>8A URDU</t>
@@ -6803,7 +6791,11 @@
           <t>6E ENGLISH</t>
         </is>
       </c>
-      <c r="O41" s="3" t="inlineStr"/>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>7D MATHS</t>
+        </is>
+      </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
           <t>6B MATHS</t>
@@ -6889,7 +6881,7 @@
       <c r="AP41" s="3" t="inlineStr"/>
       <c r="AQ41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9F GENERAL SCIENCE </t>
+          <t>9F GENERAL SCIENCE</t>
         </is>
       </c>
       <c r="AR41" s="3" t="inlineStr"/>
@@ -7112,7 +7104,11 @@
         </is>
       </c>
       <c r="AQ43" s="3" t="inlineStr"/>
-      <c r="AR43" s="3" t="inlineStr"/>
+      <c r="AR43" s="3" t="inlineStr">
+        <is>
+          <t>6A HISTORY</t>
+        </is>
+      </c>
       <c r="AS43" s="3" t="inlineStr">
         <is>
           <t>7D SINDHI</t>
@@ -7122,11 +7118,7 @@
       <c r="AU43" s="3" t="inlineStr"/>
       <c r="AV43" s="3" t="inlineStr"/>
       <c r="AW43" s="3" t="inlineStr"/>
-      <c r="AX43" s="3" t="inlineStr">
-        <is>
-          <t>6A AI</t>
-        </is>
-      </c>
+      <c r="AX43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr"/>
@@ -7267,7 +7259,11 @@
           <t>10B BIOLOGY</t>
         </is>
       </c>
-      <c r="AM44" s="2" t="inlineStr"/>
+      <c r="AM44" s="2" t="inlineStr">
+        <is>
+          <t>9A PHYSICS</t>
+        </is>
+      </c>
       <c r="AN44" s="2" t="inlineStr">
         <is>
           <t>9B BIOLOGY</t>
@@ -7279,11 +7275,7 @@
         </is>
       </c>
       <c r="AP44" s="2" t="inlineStr"/>
-      <c r="AQ44" s="2" t="inlineStr">
-        <is>
-          <t>9A CHEMISTRY</t>
-        </is>
-      </c>
+      <c r="AQ44" s="2" t="inlineStr"/>
       <c r="AR44" s="2" t="inlineStr"/>
       <c r="AS44" s="2" t="inlineStr"/>
       <c r="AT44" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Fixed login UI and Excel export bug
</commit_message>
<xml_diff>
--- a/school_timetable.xlsx
+++ b/school_timetable.xlsx
@@ -1138,7 +1138,11 @@
       </c>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>6E ENGLISH</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -1173,11 +1177,7 @@
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr"/>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>6E ARABIC</t>
-        </is>
-      </c>
+      <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr">
         <is>
@@ -1302,11 +1302,7 @@
           <t>9F URDU</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>6B ENGLISH</t>
-        </is>
-      </c>
+      <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
           <t>8D MATHS</t>
@@ -1317,7 +1313,11 @@
           <t>6A MATHS</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>6B URDU</t>
+        </is>
+      </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
           <t>7E COMPUTER</t>
@@ -1852,7 +1852,7 @@
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>6E ENGLISH</t>
+          <t>6B ENGLISH</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
@@ -1861,16 +1861,8 @@
           <t>9C MATHS</t>
         </is>
       </c>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>6B URDU</t>
-        </is>
-      </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>7A COMPUTER</t>
-        </is>
-      </c>
+      <c r="Q9" s="3" t="inlineStr"/>
+      <c r="R9" s="3" t="inlineStr"/>
       <c r="S9" s="3" t="inlineStr">
         <is>
           <t>10E COMPUTER IX-X</t>
@@ -1893,7 +1885,11 @@
           <t>10A SINDHI-X</t>
         </is>
       </c>
-      <c r="Y9" s="3" t="inlineStr"/>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>6E ARABIC</t>
+        </is>
+      </c>
       <c r="Z9" s="3" t="inlineStr"/>
       <c r="AA9" s="3" t="inlineStr">
         <is>
@@ -1931,7 +1927,11 @@
           <t>7E PH</t>
         </is>
       </c>
-      <c r="AI9" s="3" t="inlineStr"/>
+      <c r="AI9" s="3" t="inlineStr">
+        <is>
+          <t>9A LIBRARY</t>
+        </is>
+      </c>
       <c r="AJ9" s="3" t="inlineStr">
         <is>
           <t>9E PHYSICS</t>
@@ -1952,13 +1952,17 @@
           <t>10C CHEMISTRY</t>
         </is>
       </c>
-      <c r="AR9" s="3" t="inlineStr"/>
+      <c r="AR9" s="3" t="inlineStr">
+        <is>
+          <t>7A HISTORY</t>
+        </is>
+      </c>
       <c r="AS9" s="3" t="inlineStr"/>
       <c r="AT9" s="3" t="inlineStr"/>
       <c r="AU9" s="3" t="inlineStr"/>
       <c r="AV9" s="3" t="inlineStr">
         <is>
-          <t>9A GAMES</t>
+          <t>9B GAMES</t>
         </is>
       </c>
       <c r="AW9" s="3" t="inlineStr"/>
@@ -2022,7 +2026,11 @@
           <t>7E URDU</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>7A COMPUTER</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
           <t>10E COMPUTER IX-X</t>
@@ -2112,21 +2120,17 @@
         </is>
       </c>
       <c r="AQ10" s="2" t="inlineStr"/>
-      <c r="AR10" s="2" t="inlineStr">
-        <is>
-          <t>7A HISTORY</t>
-        </is>
-      </c>
+      <c r="AR10" s="2" t="inlineStr"/>
       <c r="AS10" s="2" t="inlineStr"/>
       <c r="AT10" s="2" t="inlineStr"/>
       <c r="AU10" s="2" t="inlineStr"/>
       <c r="AV10" s="2" t="inlineStr"/>
-      <c r="AW10" s="2" t="inlineStr">
-        <is>
-          <t>6B GAMES</t>
-        </is>
-      </c>
-      <c r="AX10" s="2" t="inlineStr"/>
+      <c r="AW10" s="2" t="inlineStr"/>
+      <c r="AX10" s="2" t="inlineStr">
+        <is>
+          <t>6B AI</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2781,12 +2785,12 @@
           <t>9C GAMES</t>
         </is>
       </c>
-      <c r="AW14" s="2" t="inlineStr"/>
-      <c r="AX14" s="2" t="inlineStr">
-        <is>
-          <t>6B AI</t>
-        </is>
-      </c>
+      <c r="AW14" s="2" t="inlineStr">
+        <is>
+          <t>6B GAMES</t>
+        </is>
+      </c>
+      <c r="AX14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr"/>
@@ -3714,7 +3718,11 @@
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr"/>
-      <c r="R21" s="3" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>7E COMPUTER</t>
+        </is>
+      </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
           <t>8A COMPUTER</t>
@@ -3821,11 +3829,7 @@
           <t>8B GAMES</t>
         </is>
       </c>
-      <c r="AW21" s="3" t="inlineStr">
-        <is>
-          <t>7E GAMES</t>
-        </is>
-      </c>
+      <c r="AW21" s="3" t="inlineStr"/>
       <c r="AX21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
@@ -4266,11 +4270,7 @@
       <c r="O25" s="3" t="inlineStr"/>
       <c r="P25" s="3" t="inlineStr"/>
       <c r="Q25" s="3" t="inlineStr"/>
-      <c r="R25" s="3" t="inlineStr">
-        <is>
-          <t>7E COMPUTER</t>
-        </is>
-      </c>
+      <c r="R25" s="3" t="inlineStr"/>
       <c r="S25" s="3" t="inlineStr">
         <is>
           <t>6E COMPUTER</t>
@@ -4281,7 +4281,11 @@
           <t>7C COMPUTER</t>
         </is>
       </c>
-      <c r="U25" s="3" t="inlineStr"/>
+      <c r="U25" s="3" t="inlineStr">
+        <is>
+          <t>9A ENGLISH</t>
+        </is>
+      </c>
       <c r="V25" s="3" t="inlineStr"/>
       <c r="W25" s="3" t="inlineStr">
         <is>
@@ -4323,11 +4327,7 @@
       </c>
       <c r="AG25" s="3" t="inlineStr"/>
       <c r="AH25" s="3" t="inlineStr"/>
-      <c r="AI25" s="3" t="inlineStr">
-        <is>
-          <t>9A LIBRARY</t>
-        </is>
-      </c>
+      <c r="AI25" s="3" t="inlineStr"/>
       <c r="AJ25" s="3" t="inlineStr">
         <is>
           <t>10E PHYSICS</t>
@@ -4373,7 +4373,11 @@
           <t>8D GAMES</t>
         </is>
       </c>
-      <c r="AW25" s="3" t="inlineStr"/>
+      <c r="AW25" s="3" t="inlineStr">
+        <is>
+          <t>7E GAMES</t>
+        </is>
+      </c>
       <c r="AX25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
@@ -4441,11 +4445,7 @@
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr">
-        <is>
-          <t>9A ENGLISH</t>
-        </is>
-      </c>
+      <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="inlineStr">
         <is>
           <t>8B ENGLISH</t>
@@ -4536,7 +4536,11 @@
       </c>
       <c r="AT26" s="2" t="inlineStr"/>
       <c r="AU26" s="2" t="inlineStr"/>
-      <c r="AV26" s="2" t="inlineStr"/>
+      <c r="AV26" s="2" t="inlineStr">
+        <is>
+          <t>9A GAMES</t>
+        </is>
+      </c>
       <c r="AW26" s="2" t="inlineStr"/>
       <c r="AX26" s="2" t="inlineStr"/>
     </row>
@@ -5376,11 +5380,7 @@
           <t>10:40-11:15</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>6A ENGLISH</t>
-        </is>
-      </c>
+      <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -5422,7 +5422,11 @@
       <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
       <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>6A COMPUTER</t>
+        </is>
+      </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
           <t>7D COMPUTER</t>
@@ -5762,7 +5766,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>7D ENGLISH</t>
+          <t>6A ENGLISH</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -5806,11 +5810,7 @@
           <t>7E URDU</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>6A COMPUTER</t>
-        </is>
-      </c>
+      <c r="R35" s="3" t="inlineStr"/>
       <c r="S35" s="3" t="inlineStr">
         <is>
           <t>8A COMPUTER</t>
@@ -5909,7 +5909,11 @@
       <c r="AT35" s="3" t="inlineStr"/>
       <c r="AU35" s="3" t="inlineStr"/>
       <c r="AV35" s="3" t="inlineStr"/>
-      <c r="AW35" s="3" t="inlineStr"/>
+      <c r="AW35" s="3" t="inlineStr">
+        <is>
+          <t>7D GAMES</t>
+        </is>
+      </c>
       <c r="AX35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
@@ -5983,11 +5987,7 @@
         </is>
       </c>
       <c r="V36" s="2" t="inlineStr"/>
-      <c r="W36" s="2" t="inlineStr">
-        <is>
-          <t>7D ISLAMIAT</t>
-        </is>
-      </c>
+      <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr">
         <is>
           <t>10C SINDHI-X</t>
@@ -6069,7 +6069,11 @@
           <t>6B HISTORY</t>
         </is>
       </c>
-      <c r="AS36" s="2" t="inlineStr"/>
+      <c r="AS36" s="2" t="inlineStr">
+        <is>
+          <t>7D SINDHI</t>
+        </is>
+      </c>
       <c r="AT36" s="2" t="inlineStr"/>
       <c r="AU36" s="2" t="inlineStr"/>
       <c r="AV36" s="2" t="inlineStr"/>
@@ -6088,7 +6092,11 @@
           <t>1:15-2:00</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>7D ENGLISH</t>
+        </is>
+      </c>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
@@ -6233,11 +6241,7 @@
       <c r="AT37" s="3" t="inlineStr"/>
       <c r="AU37" s="3" t="inlineStr"/>
       <c r="AV37" s="3" t="inlineStr"/>
-      <c r="AW37" s="3" t="inlineStr">
-        <is>
-          <t>7D GAMES</t>
-        </is>
-      </c>
+      <c r="AW37" s="3" t="inlineStr"/>
       <c r="AX37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -6294,7 +6298,11 @@
           <t>8C URDU</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>7E ENGLISH</t>
+        </is>
+      </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
           <t>8D MATHS</t>
@@ -6333,11 +6341,7 @@
           <t>10E SINDHI-X</t>
         </is>
       </c>
-      <c r="Y38" s="2" t="inlineStr">
-        <is>
-          <t>7E ARABIC</t>
-        </is>
-      </c>
+      <c r="Y38" s="2" t="inlineStr"/>
       <c r="Z38" s="2" t="inlineStr">
         <is>
           <t>9D ISLAMIAT IX</t>
@@ -6458,11 +6462,7 @@
           <t>9F URDU</t>
         </is>
       </c>
-      <c r="N39" s="3" t="inlineStr">
-        <is>
-          <t>7E ENGLISH</t>
-        </is>
-      </c>
+      <c r="N39" s="3" t="inlineStr"/>
       <c r="O39" s="3" t="inlineStr">
         <is>
           <t>8D MATHS</t>
@@ -6497,7 +6497,11 @@
         </is>
       </c>
       <c r="X39" s="3" t="inlineStr"/>
-      <c r="Y39" s="3" t="inlineStr"/>
+      <c r="Y39" s="3" t="inlineStr">
+        <is>
+          <t>7E ARABIC</t>
+        </is>
+      </c>
       <c r="Z39" s="3" t="inlineStr">
         <is>
           <t>9A ISLAMIAT IX</t>
@@ -7043,7 +7047,11 @@
       </c>
       <c r="U43" s="3" t="inlineStr"/>
       <c r="V43" s="3" t="inlineStr"/>
-      <c r="W43" s="3" t="inlineStr"/>
+      <c r="W43" s="3" t="inlineStr">
+        <is>
+          <t>7D ISLAMIAT</t>
+        </is>
+      </c>
       <c r="X43" s="3" t="inlineStr">
         <is>
           <t>8C SINDHI</t>
@@ -7109,11 +7117,7 @@
           <t>6A HISTORY</t>
         </is>
       </c>
-      <c r="AS43" s="3" t="inlineStr">
-        <is>
-          <t>7D SINDHI</t>
-        </is>
-      </c>
+      <c r="AS43" s="3" t="inlineStr"/>
       <c r="AT43" s="3" t="inlineStr"/>
       <c r="AU43" s="3" t="inlineStr"/>
       <c r="AV43" s="3" t="inlineStr"/>

</xml_diff>